<commit_message>
Ultima actualizacion inventarios  sst, locativo y sistemas
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Proyectos\crm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326D5947-7BD2-4359-8DF8-74708F72B3ED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A1B864-2BAC-464A-982E-2C4635B7C48F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{AA60AC60-657F-41AC-8562-B66377B22196}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$L$494</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$L$495</definedName>
   </definedNames>
   <calcPr calcId="179021"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="194">
   <si>
     <t>Nombre</t>
   </si>
@@ -607,6 +607,9 @@
   </si>
   <si>
     <t>BL 27 LAS MALVINAS CENTRAL MAYORISTA</t>
+  </si>
+  <si>
+    <t>Cll 31 # 41 51</t>
   </si>
 </sst>
 </file>
@@ -959,7 +962,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB89B2D1-2EEC-48D7-ADDC-0BC745E25224}">
-  <dimension ref="A1:L494"/>
+  <dimension ref="A1:L495"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1000,18 +1003,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" t="s">
-        <v>25</v>
+    <row r="2" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <v>890919352</v>
+      </c>
+      <c r="C2" s="1">
+        <v>6044447773</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>
@@ -1026,21 +1026,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
@@ -1054,16 +1054,16 @@
     </row>
     <row r="4" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
         <v>12</v>
@@ -1078,18 +1078,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -1097,9 +1097,6 @@
       <c r="F5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
       <c r="J5" t="s">
         <v>14</v>
       </c>
@@ -1109,16 +1106,16 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -1138,16 +1135,16 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
         <v>12</v>
@@ -1167,16 +1164,16 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>
@@ -1196,16 +1193,16 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
         <v>12</v>
@@ -1225,19 +1222,19 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
@@ -1254,16 +1251,16 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
         <v>18</v>
@@ -1283,19 +1280,19 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>13</v>
@@ -1312,19 +1309,19 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
@@ -1341,19 +1338,19 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>13</v>
@@ -1370,19 +1367,19 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>13</v>
@@ -1399,19 +1396,19 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D16" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>13</v>
@@ -1428,19 +1425,19 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>13</v>
@@ -1457,19 +1454,19 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
@@ -1486,16 +1483,16 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B19" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E19" t="s">
         <v>12</v>
@@ -1515,19 +1512,19 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>13</v>
@@ -1544,19 +1541,19 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D21" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>13</v>
@@ -1573,16 +1570,16 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B22" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E22" t="s">
         <v>12</v>
@@ -1602,19 +1599,19 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D23" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>13</v>
@@ -1631,19 +1628,19 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D24" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E24" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>13</v>
@@ -1660,16 +1657,16 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B25" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E25" t="s">
         <v>12</v>
@@ -1689,19 +1686,19 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E26" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>13</v>
@@ -1718,19 +1715,19 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>17</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E27" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>13</v>
@@ -1747,16 +1744,16 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E28" t="s">
         <v>12</v>
@@ -1776,19 +1773,19 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B29" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C29" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>13</v>
@@ -1805,19 +1802,19 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>131</v>
       </c>
       <c r="D30" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="E30" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>13</v>
@@ -1834,16 +1831,16 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B31" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C31" t="s">
-        <v>137</v>
+        <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>138</v>
+        <v>17</v>
       </c>
       <c r="E31" t="s">
         <v>18</v>
@@ -1863,19 +1860,19 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B32" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C32" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D32" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>13</v>
@@ -1892,19 +1889,19 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C33" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D33" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E33" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>13</v>
@@ -1921,19 +1918,19 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B34" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C34" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E34" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
@@ -1950,19 +1947,19 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B35" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>149</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
+        <v>150</v>
       </c>
       <c r="E35" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
@@ -1979,19 +1976,19 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B36" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>17</v>
       </c>
       <c r="D36" t="s">
-        <v>156</v>
+        <v>17</v>
       </c>
       <c r="E36" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -2008,16 +2005,16 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B37" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C37" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D37" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E37" t="s">
         <v>12</v>
@@ -2037,16 +2034,16 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B38" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D38" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E38" t="s">
         <v>12</v>
@@ -2066,16 +2063,16 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B39" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C39" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D39" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E39" t="s">
         <v>12</v>
@@ -2095,16 +2092,16 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B40" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C40" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D40" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E40" t="s">
         <v>12</v>
@@ -2124,19 +2121,19 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B41" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C41" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D41" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E41" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>13</v>
@@ -2153,19 +2150,19 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B42" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C42" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D42" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E42" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>13</v>
@@ -2182,19 +2179,19 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B43" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C43" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D43" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E43" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>13</v>
@@ -2211,19 +2208,19 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C44" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D44" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E44" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>13</v>
@@ -2240,16 +2237,16 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B45" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C45" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D45" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E45" t="s">
         <v>18</v>
@@ -2267,13 +2264,34 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46"/>
-      <c r="B46"/>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="J46"/>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" t="s">
+        <v>190</v>
+      </c>
+      <c r="C46" t="s">
+        <v>191</v>
+      </c>
+      <c r="D46" t="s">
+        <v>192</v>
+      </c>
+      <c r="E46" t="s">
+        <v>18</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="1"/>
+      <c r="J46" t="s">
+        <v>14</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="47" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47"/>
@@ -5859,6 +5877,14 @@
       <c r="E494"/>
       <c r="J494"/>
     </row>
+    <row r="495" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A495"/>
+      <c r="B495"/>
+      <c r="C495"/>
+      <c r="D495"/>
+      <c r="E495"/>
+      <c r="J495"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>